<commit_message>
added horizontal scrolling on top
</commit_message>
<xml_diff>
--- a/docs/03-Component-Selection/Power_Budget.xlsx
+++ b/docs/03-Component-Selection/Power_Budget.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\college\sp26\egr314\botilarm.github.io\docs\03-Component-Selection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1415FA1-9733-46E0-B2F7-0B00EE4F2BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16BF281-35FE-4EBE-9B7A-AC149C5FB90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="670" yWindow="-110" windowWidth="18640" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="-120" windowWidth="28170" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Budget" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="81">
   <si>
     <t>Team Number:</t>
   </si>
@@ -204,9 +204,6 @@
     <t>SER0039</t>
   </si>
   <si>
-    <t>SM-42HB34F08AB</t>
-  </si>
-  <si>
     <t xml:space="preserve">9G RC Servo </t>
   </si>
   <si>
@@ -216,9 +213,6 @@
     <t>Stepper motor driver</t>
   </si>
   <si>
-    <t>TMC260C-PA</t>
-  </si>
-  <si>
     <t>LTST-M670TBKT</t>
   </si>
   <si>
@@ -301,6 +295,18 @@
   </si>
   <si>
     <t>+0-57V</t>
+  </si>
+  <si>
+    <t>TMC2209-LA-T</t>
+  </si>
+  <si>
+    <t>+4.8V - 5.25V</t>
+  </si>
+  <si>
+    <t>FIT0278</t>
+  </si>
+  <si>
+    <t>+3.4V</t>
   </si>
 </sst>
 </file>
@@ -580,7 +586,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -725,6 +731,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -734,7 +755,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -750,19 +770,8 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1114,31 +1123,31 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H59"/>
-  <sheetFormatPr defaultColWidth="13.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="13.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="33.58203125" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="33.625" customWidth="1"/>
+    <col min="3" max="3" width="22.375" customWidth="1"/>
     <col min="4" max="4" width="30.75" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="6" width="38.1640625" customWidth="1"/>
+    <col min="6" max="6" width="38.125" customWidth="1"/>
     <col min="7" max="7" width="31.75" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="71" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+    </row>
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1148,7 +1157,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1162,7 +1171,7 @@
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="46" t="s">
         <v>2</v>
       </c>
@@ -1176,7 +1185,7 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1190,7 +1199,7 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1200,8 +1209,8 @@
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="67" t="s">
+    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="73" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -1226,16 +1235,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="67"/>
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="73"/>
       <c r="B8" s="52" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>45</v>
       </c>
       <c r="D8" s="54" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E8" s="49">
         <v>3</v>
@@ -1251,41 +1260,41 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="67"/>
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="73"/>
       <c r="B9" s="52" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="52" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="D9" s="54" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E9" s="49">
         <v>1</v>
       </c>
       <c r="F9" s="52">
-        <v>1330</v>
+        <v>1700</v>
       </c>
       <c r="G9" s="51">
         <f t="shared" si="0"/>
-        <v>1330</v>
+        <v>1700</v>
       </c>
       <c r="H9" s="51" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="67"/>
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="73"/>
       <c r="B10" s="52" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C10" s="52" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="D10" s="54" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="49">
         <v>1</v>
@@ -1301,16 +1310,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="67"/>
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="73"/>
       <c r="B11" s="52" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C11" s="52" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D11" s="56" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E11" s="49">
         <v>5</v>
@@ -1326,16 +1335,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="67"/>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="73"/>
       <c r="B12" s="52" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C12" s="52" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" s="54" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E12" s="49">
         <v>1</v>
@@ -1351,7 +1360,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="15"/>
       <c r="D13" s="11"/>
@@ -1359,7 +1368,7 @@
       <c r="G13" s="13"/>
       <c r="H13" s="14"/>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="5"/>
       <c r="C14" s="4"/>
@@ -1369,8 +1378,8 @@
       <c r="G14" s="18"/>
       <c r="H14" s="18"/>
     </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="68" t="s">
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="74" t="s">
         <v>15</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -1395,80 +1404,80 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="68"/>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="74"/>
       <c r="B16" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="52" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="D16" s="54" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E16" s="12">
         <v>1</v>
       </c>
       <c r="F16">
-        <v>1330</v>
+        <v>1700</v>
       </c>
       <c r="G16" s="13">
         <f t="shared" ref="G16" si="1">E16*F16</f>
-        <v>1330</v>
+        <v>1700</v>
       </c>
       <c r="H16" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="68"/>
-      <c r="B17" s="66" t="s">
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="74"/>
+      <c r="B17" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="65"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="65"/>
-      <c r="F17" s="65"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="63"/>
       <c r="G17" s="13">
         <f>SUM(G16:G16)</f>
-        <v>1330</v>
+        <v>1700</v>
       </c>
       <c r="H17" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="68"/>
-      <c r="B18" s="66" t="s">
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="74"/>
+      <c r="B18" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="65"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="65"/>
-      <c r="F18" s="65"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
       <c r="G18" s="21">
         <v>0.25</v>
       </c>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
-      <c r="B19" s="69" t="s">
+      <c r="B19" s="75" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="65"/>
-      <c r="D19" s="65"/>
-      <c r="E19" s="65"/>
-      <c r="F19" s="65"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="63"/>
       <c r="G19" s="13">
         <f>G17*(1+G18)</f>
-        <v>1662.5</v>
+        <v>2125</v>
       </c>
       <c r="H19" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="23"/>
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
@@ -1478,40 +1487,41 @@
       <c r="G20" s="26"/>
       <c r="H20" s="13"/>
     </row>
-    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="53" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C21" s="24"/>
       <c r="D21" s="49" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E21" s="11">
         <v>1</v>
       </c>
       <c r="F21" s="25">
-        <v>1662.5</v>
+        <f>G19</f>
+        <v>2125</v>
       </c>
       <c r="G21" s="26">
         <f>E21*F21</f>
-        <v>1662.5</v>
+        <v>2125</v>
       </c>
       <c r="H21" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="23"/>
-      <c r="B22" s="70" t="s">
+      <c r="B22" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="71"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="71"/>
-      <c r="F22" s="71"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="66"/>
       <c r="G22" s="26">
         <f>G21-G19</f>
         <v>0</v>
@@ -1520,8 +1530,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="62" t="s">
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="69" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -1546,16 +1556,16 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="63"/>
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="70"/>
       <c r="B24" s="52" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" s="52" t="s">
         <v>45</v>
       </c>
       <c r="D24" s="50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E24" s="12">
         <v>3</v>
@@ -1571,169 +1581,166 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="63"/>
-      <c r="B25" s="66" t="s">
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="70"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="77" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="12">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>25</v>
+      </c>
+      <c r="G25" s="13">
+        <v>25</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="70"/>
+      <c r="B26" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="65"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="65"/>
-      <c r="G25" s="13">
-        <f>SUM(G24:G24)</f>
-        <v>900</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="63"/>
-      <c r="B26" s="66" t="s">
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
+      <c r="E26" s="63"/>
+      <c r="F26" s="63"/>
+      <c r="G26" s="13">
+        <f>SUM(G24:G25)</f>
+        <v>925</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="70"/>
+      <c r="B27" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="65"/>
-      <c r="D26" s="65"/>
-      <c r="E26" s="65"/>
-      <c r="F26" s="65"/>
-      <c r="G26" s="21">
+      <c r="C27" s="63"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="63"/>
+      <c r="F27" s="63"/>
+      <c r="G27" s="21">
         <v>0.25</v>
       </c>
-      <c r="H26" s="21"/>
-    </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="22"/>
-      <c r="B27" s="69" t="s">
+      <c r="H27" s="21"/>
+    </row>
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22"/>
+      <c r="B28" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="C27" s="65"/>
-      <c r="D27" s="65"/>
-      <c r="E27" s="65"/>
-      <c r="F27" s="65"/>
-      <c r="G27" s="13">
-        <f>G25*(1+G26)</f>
-        <v>1125</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="23"/>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="13"/>
-    </row>
-    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="23" t="s">
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="63"/>
+      <c r="G28" s="13">
+        <f>G26*(1+G27)</f>
+        <v>1156.25</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="23"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="13"/>
+    </row>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="53" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="D29" s="54" t="s">
-        <v>78</v>
-      </c>
-      <c r="E29" s="11">
+      <c r="B30" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="54" t="s">
+        <v>76</v>
+      </c>
+      <c r="E30" s="11">
         <v>1</v>
       </c>
-      <c r="F29" s="25">
+      <c r="F30" s="25">
         <v>2000</v>
       </c>
-      <c r="G29" s="26">
-        <f>E29*F29</f>
+      <c r="G30" s="26">
+        <f>E30*F30</f>
         <v>2000</v>
       </c>
-      <c r="H29" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="23"/>
-      <c r="B30" s="70" t="s">
+      <c r="H30" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="23"/>
+      <c r="B31" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-      <c r="F30" s="71"/>
-      <c r="G30" s="26">
-        <f>G29-G27</f>
-        <v>875</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="62" t="s">
+      <c r="C31" s="66"/>
+      <c r="D31" s="66"/>
+      <c r="E31" s="66"/>
+      <c r="F31" s="66"/>
+      <c r="G31" s="26">
+        <f>G30-G28</f>
+        <v>843.75</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B32" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C32" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D32" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E32" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F32" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G31" s="28" t="s">
+      <c r="G32" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="H31" s="28" t="s">
+      <c r="H32" s="28" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="63"/>
-      <c r="B32" s="52" t="s">
-        <v>49</v>
-      </c>
-      <c r="C32" s="52" t="s">
-        <v>50</v>
-      </c>
-      <c r="D32" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="E32" s="12">
-        <v>1</v>
-      </c>
-      <c r="F32" s="15">
-        <v>12</v>
-      </c>
-      <c r="G32" s="14">
-        <f>F32*E32</f>
-        <v>12</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="63"/>
+    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="70"/>
       <c r="B33" s="52" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C33" s="52" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D33" s="54" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E33" s="12">
         <v>1</v>
@@ -1749,16 +1756,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="63"/>
+    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="70"/>
       <c r="B34" s="52" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C34" s="52" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D34" s="56" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E34" s="12">
         <v>5</v>
@@ -1774,55 +1781,55 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="63"/>
-      <c r="B35" s="66" t="s">
+    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="70"/>
+      <c r="B35" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="C35" s="65"/>
-      <c r="D35" s="65"/>
-      <c r="E35" s="65"/>
-      <c r="F35" s="65"/>
+      <c r="C35" s="63"/>
+      <c r="D35" s="63"/>
+      <c r="E35" s="63"/>
+      <c r="F35" s="63"/>
       <c r="G35" s="13">
-        <f>SUM(G31:G34)</f>
-        <v>467</v>
+        <f>SUM(G32:G34)</f>
+        <v>455</v>
       </c>
       <c r="H35" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="63"/>
-      <c r="B36" s="66" t="s">
+    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="70"/>
+      <c r="B36" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="C36" s="65"/>
-      <c r="D36" s="65"/>
-      <c r="E36" s="65"/>
-      <c r="F36" s="65"/>
+      <c r="C36" s="63"/>
+      <c r="D36" s="63"/>
+      <c r="E36" s="63"/>
+      <c r="F36" s="63"/>
       <c r="G36" s="21">
         <v>0.25</v>
       </c>
       <c r="H36" s="21"/>
     </row>
-    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
-      <c r="B37" s="72" t="s">
+      <c r="B37" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="65"/>
-      <c r="D37" s="65"/>
-      <c r="E37" s="65"/>
-      <c r="F37" s="65"/>
+      <c r="C37" s="63"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="63"/>
+      <c r="F37" s="63"/>
       <c r="G37" s="13">
         <f>G35*(1+G36)</f>
-        <v>583.75</v>
+        <v>568.75</v>
       </c>
       <c r="H37" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23"/>
       <c r="B38" s="24"/>
       <c r="C38" s="24"/>
@@ -1832,18 +1839,18 @@
       <c r="G38" s="26"/>
       <c r="H38" s="13"/>
     </row>
-    <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="23" t="s">
         <v>25</v>
       </c>
       <c r="B39" s="55" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C39" s="24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D39" s="54" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E39" s="11">
         <v>1</v>
@@ -1859,24 +1866,24 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="27"/>
-      <c r="B40" s="73" t="s">
-        <v>68</v>
-      </c>
-      <c r="C40" s="71"/>
-      <c r="D40" s="71"/>
-      <c r="E40" s="71"/>
-      <c r="F40" s="71"/>
+      <c r="B40" s="65" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="66"/>
+      <c r="D40" s="66"/>
+      <c r="E40" s="66"/>
+      <c r="F40" s="66"/>
       <c r="G40" s="26">
         <f>G39-G37</f>
-        <v>416.25</v>
+        <v>431.25</v>
       </c>
       <c r="H40" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
         <v>28</v>
       </c>
@@ -1902,21 +1909,21 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="30" t="s">
         <v>30</v>
       </c>
       <c r="B42" s="53" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C42" s="49" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E42" s="58" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F42" s="25">
         <v>5000</v>
@@ -1929,7 +1936,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="33"/>
       <c r="B43" s="24"/>
       <c r="C43" s="24"/>
@@ -1939,21 +1946,21 @@
       <c r="G43" s="26"/>
       <c r="H43" s="34"/>
     </row>
-    <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="74" t="s">
+    <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="67" t="s">
         <v>31</v>
       </c>
       <c r="B44" s="57" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C44" s="49" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D44" s="49" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E44" s="58" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F44" s="25">
         <v>1662.5</v>
@@ -1966,19 +1973,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="75"/>
+    <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="68"/>
       <c r="B45" s="24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C45" s="24" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D45" s="54" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E45" s="58" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F45" s="25">
         <v>2000</v>
@@ -1991,19 +1998,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="75"/>
+    <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="68"/>
       <c r="B46" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C46" s="24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D46" s="54" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E46" s="61" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F46">
         <v>1000</v>
@@ -2016,15 +2023,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="33"/>
-      <c r="B47" s="76" t="s">
+      <c r="B47" s="62" t="s">
         <v>32</v>
       </c>
-      <c r="C47" s="65"/>
-      <c r="D47" s="65"/>
-      <c r="E47" s="65"/>
-      <c r="F47" s="65"/>
+      <c r="C47" s="63"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="63"/>
+      <c r="F47" s="63"/>
       <c r="G47" s="31">
         <f>G42-SUM(G44:G46)</f>
         <v>337.5</v>
@@ -2033,7 +2040,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="33"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -2043,7 +2050,7 @@
       <c r="G48" s="35"/>
       <c r="H48" s="36"/>
     </row>
-    <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="19" t="s">
         <v>33</v>
       </c>
@@ -2069,19 +2076,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="30" t="s">
         <v>34</v>
       </c>
       <c r="B50" s="57" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C50" s="58"/>
       <c r="D50" s="59" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E50" s="59" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F50" s="60">
         <v>5000</v>
@@ -2094,7 +2101,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="33"/>
       <c r="B51" s="24"/>
       <c r="C51" s="24"/>
@@ -2104,21 +2111,21 @@
       <c r="G51" s="26"/>
       <c r="H51" s="34"/>
     </row>
-    <row r="52" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="74" t="s">
+    <row r="52" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="67" t="s">
         <v>36</v>
       </c>
       <c r="B52" s="57" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C52" s="49" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D52" s="49" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E52" s="58" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F52" s="25">
         <v>1662.5</v>
@@ -2131,19 +2138,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="75"/>
+    <row r="53" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="68"/>
       <c r="B53" s="24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C53" s="24" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D53" s="54" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E53" s="58" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F53" s="25">
         <v>2000</v>
@@ -2156,19 +2163,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="75"/>
+    <row r="54" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="68"/>
       <c r="B54" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C54" s="24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D54" s="54" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E54" s="61" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F54">
         <v>1000</v>
@@ -2181,15 +2188,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="33"/>
-      <c r="B55" s="76" t="s">
+      <c r="B55" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="C55" s="65"/>
-      <c r="D55" s="65"/>
-      <c r="E55" s="65"/>
-      <c r="F55" s="65"/>
+      <c r="C55" s="63"/>
+      <c r="D55" s="63"/>
+      <c r="E55" s="63"/>
+      <c r="F55" s="63"/>
       <c r="G55" s="31">
         <f>G50-SUM(G52:G54)</f>
         <v>337.5</v>
@@ -2198,7 +2205,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="22"/>
       <c r="B56" s="15"/>
       <c r="D56" s="37"/>
@@ -2207,7 +2214,7 @@
       <c r="G56" s="13"/>
       <c r="H56" s="38"/>
     </row>
-    <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="39"/>
       <c r="B57" s="40" t="s">
         <v>5</v>
@@ -2227,7 +2234,7 @@
       </c>
       <c r="H57" s="44"/>
     </row>
-    <row r="58" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
       <c r="B58" t="s">
         <v>35</v>
@@ -2248,7 +2255,7 @@
       </c>
       <c r="H58" s="13"/>
     </row>
-    <row r="59" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="10"/>
       <c r="D59" s="12"/>
       <c r="E59" s="12"/>
@@ -2265,14 +2272,8 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B55:F55"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="A52:A54"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A31:A36"/>
+    <mergeCell ref="A23:A27"/>
+    <mergeCell ref="A32:A36"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B18:F18"/>
@@ -2280,14 +2281,20 @@
     <mergeCell ref="A15:A18"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B25:F25"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B31:F31"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="A52:A54"/>
   </mergeCells>
-  <conditionalFormatting sqref="G22 G30 G40">
+  <conditionalFormatting sqref="G22 G31 G40">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>